<commit_message>
ci: regenera página y Excel
</commit_message>
<xml_diff>
--- a/docs/research.xlsx
+++ b/docs/research.xlsx
@@ -31,7 +31,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'training'!$A$1:$W$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'watchlist_closed'!$A$1:$L$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'subscriptions'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'sources'!$A$1:$J$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'sources'!$A$1:$J$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'inbox_triage'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'changelog'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'readme'!$A$1:$B$33</definedName>
@@ -542,11 +542,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
@@ -637,7 +637,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>research field: genetics/statistics OR neuroscience OR psychiatry; country: all EU/EEA; keywords "statistical genetics", "GWAS", "polygenic risk score", "psychiatric genetics", "sleep genetics"</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -653,7 +653,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>subject: Biological Sciences / Psychology; keywords "statistical genetics", "psychiatric genetics", "GWAS", "PRS", "behavioural genetics", "sleep"</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -701,7 +701,7 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>keywords "statistical genetics", "GWAS", "polygenic risk score", "psychiatric genetics", "behavioural genetics", "sleep genetics"; all countries</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -749,7 +749,7 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>keywords "statistical genetics", "psychiatric genetics", "GWAS", "PRS", "computational genetics"</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -797,7 +797,7 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>field: Genetics / Neuroscience / Psychology; keywords "statistical genetics", "psychiatric genetics", "GWAS", "PRS"</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -845,7 +845,7 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>keywords "statistical genetics", "psychiatric genetics", "GWAS", "PRS", "sleep genetics", "behavioural genetics"</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -893,7 +893,7 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>keywords "statistical genetics", "genetic epidemiology", "sleep genetics" — the Netherlands is a hub for both (Erasmus MC, VU Netherlands Twin Register)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -941,7 +941,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>keywords "statistical genetics", "psychiatric genetics", "GWAS", "PRS", "behavioural genetics"</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -989,7 +989,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[TODO: titulos de rol segun perfil]</t>
+          <t>titles: "statistical geneticist", "computational genetics", "genetic epidemiologist", "medical science liaison", "medical writer", "science communication officer"; countries: EU/EEA, Australia, USA, UK and other English-speaking, remote included</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1037,7 +1037,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>keywords "statistical genetics", "computational biology", "genomics", "clinical genetics"; companies of interest: 23andMe, Invitae, Color Health, Genomics England, Regeneron Genetics Center, Illumina, deCODE genetics</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>annual call page + open calendar</t>
+          <t>annual call page + open calendar; verify mobility rule against her Spain/Australia/Japan last-3-years residence</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1133,7 +1133,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>rolling; check eligibility window</t>
+          <t>rolling; check eligibility window against Feb 2028 (ETA) defense date</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1181,7 +1181,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>annual call page</t>
+          <t>annual call page; cross-disciplinary angle (genetics + neuroscience) is a good fit</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1229,7 +1229,7 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[TODO: mantener solo si España/Portugal entra en juego]</t>
+          <t>Junior Leader Incoming/Retaining calls; Spain is home base, keep in play</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1277,7 +1277,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>[TODO: mantener solo si España entra en juego]</t>
+          <t>Sara Borrell y Rio Hortega (postdoc temprano); Miguel Servet (mas senior, vigilar plazo); España sigue en juego</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1325,7 +1325,7 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>[TODO: mantener solo si España entra en juego]</t>
+          <t>Juan de la Cierva Formación/Incorporación y Ramón y Cajal; España sigue en juego</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1373,7 +1373,7 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>[TODO: mantener solo si Alemania entra en juego]</t>
+          <t>Alemania esta en juego (UE/EEE sin exclusiones); rolling postdoc fellowships</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1421,7 +1421,7 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>[TODO: mantener solo si UK entra en juego]</t>
+          <t>Reino Unido esta en juego (angloparlante YES); relevante por los hubs de genetica psiquiatrica (King's, Cardiff, Edinburgh)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1469,7 +1469,7 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>jobs + training + kavli network</t>
+          <t>jobs + training + kavli network; keywords behavioural/cognitive neuroscience</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1517,7 +1517,7 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>schools and grants relevant to behavioural/cognitive neuroscience and to her Japan-stay skill set (electrophysiology/optogenetics)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1565,7 +1565,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1661,7 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>keywords "statistical genetics", "GWAS", "PRS", "sleep", "electrophysiology"</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1709,7 +1709,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[TODO: afinar query al perfil]</t>
+          <t>keywords "statistical genetics", "genomics", "computational neuroscience"</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1757,7 +1757,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[TODO: paneles LS segun perfil]</t>
+          <t>panel LS2 (Genetics, Genomics, Bioinformatics) and LS5 (Neuroscience/Neurology/Psychiatry)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1805,12 +1805,204 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>semilla 2026-08-23; revisar cuando el perfil este definido</t>
+          <t>afinada tras definir el perfil, 2026-08-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SRC-0026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>World Congress of Psychiatric Genetics (WCPG)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>EVENTS</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://worldcongressofpsychiatricgenetics.org</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Central annual venue for GWAS/PRS psychiatric genetics: dates, abstract deadline, travel awards</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>abstract deadline + travel award programme</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>añadida tras definir el perfil, 2026-08-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SRC-0027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Psychiatric Genomics Consortium (PGC)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>GROUPS</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://pgc.unc.edu</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Working-group membership and activity map for GWAS/PRS psychiatric genetics; occasional analyst/training openings</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>working group pages by disorder; new working-group calls</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>añadida tras definir el perfil, 2026-08-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SRC-0028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Boletín Oficial del Estado (BOE) — especialidad de Genética</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>JOBS</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.boe.es</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Real decreto y desarrollo de la via transitoria de la especialidad de Genetica Medica y de Laboratorio</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>buscar "Genética Médica y de Laboratorio", "vía transitoria", "real decreto especialidad"</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>añadida tras definir el perfil, 2026-08-23; carril B, primera clase</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SRC-0029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bolsas/oposiciones de Genética por Comunidad Autónoma</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>JOBS</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>[TODO: una URL por CCAA — servicio de salud de cada comunidad]</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Convocatorias de facultativo especialista en Genética/Análisis Clínicos por CCAA (bolsa de empleo, oposición o concurso: mecanismo distinto por comunidad)</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>revisar cada portal de salud autonómico por separado; empezar por Andalucía (SAS, dado el destino de la residencia en Málaga) y ampliar</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>añadida tras definir el perfil, 2026-08-23; carril B, primera clase — URLs por CCAA pendientes de completar en la primera pasada</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J26"/>
+  <autoFilter ref="A1:J30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>